<commit_message>
Daily freezer layout export
</commit_message>
<xml_diff>
--- a/cellstocks/exports/layout.xlsx
+++ b/cellstocks/exports/layout.xlsx
@@ -3,13 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="boxes" sheetId="1" r:id="rId1"/>
-    <sheet name="Baro CELLS #1 (-80)" sheetId="2" r:id="rId2"/>
-    <sheet name="UMUT CAA CELLS" sheetId="3" r:id="rId3"/>
-    <sheet name="UMUT CELLS -80" sheetId="4" r:id="rId4"/>
-    <sheet name="DUZENLE" sheetId="5" r:id="rId5"/>
-    <sheet name="ONGOING" sheetId="6" r:id="rId6"/>
-    <sheet name="UMUT CELLS -4-" sheetId="7" r:id="rId7"/>
-    <sheet name="Unnamed box" sheetId="8" r:id="rId8"/>
+    <sheet name="UMUT CAA CELLS" sheetId="2" r:id="rId2"/>
+    <sheet name="UMUT CELLS -80" sheetId="3" r:id="rId3"/>
+    <sheet name="DUZENLE" sheetId="4" r:id="rId4"/>
+    <sheet name="ONGOING" sheetId="5" r:id="rId5"/>
+    <sheet name="UMUT CELLS -4-" sheetId="6" r:id="rId6"/>
+    <sheet name="Unnamed box" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -105,22 +104,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baro CELLS #1 (-80)</t>
+          <t xml:space="preserve">UMUT CAA CELLS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">baris</t>
+          <t xml:space="preserve">umut</t>
         </is>
       </c>
       <c r="E2">
@@ -130,29 +129,29 @@
         <v>9</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="H2">
         <v>81</v>
       </c>
       <c r="I2">
-        <v>81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CAA CELLS</t>
+          <t xml:space="preserve">UMUT CELLS -80</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -179,17 +178,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -80</t>
+          <t xml:space="preserve">DUZENLE</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -204,29 +203,29 @@
         <v>9</v>
       </c>
       <c r="G4">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="H4">
         <v>81</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DUZENLE</t>
+          <t xml:space="preserve">ONGOING</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -241,29 +240,29 @@
         <v>9</v>
       </c>
       <c r="G5">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H5">
         <v>81</v>
       </c>
       <c r="I5">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ONGOING</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -278,29 +277,29 @@
         <v>9</v>
       </c>
       <c r="G6">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="H6">
         <v>81</v>
       </c>
       <c r="I6">
-        <v>5</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-</t>
+          <t xml:space="preserve">Unnamed box</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -315,49 +314,12 @@
         <v>9</v>
       </c>
       <c r="G7">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H7">
         <v>81</v>
       </c>
       <c r="I7">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not placed yet</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not placed yet</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unnamed box</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">umut</t>
-        </is>
-      </c>
-      <c r="E8">
-        <v>9</v>
-      </c>
-      <c r="F8">
-        <v>9</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>81</v>
-      </c>
-      <c r="I8">
         <v>81</v>
       </c>
     </row>
@@ -371,14 +333,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baro CELLS #1 (-80)  ·  baris  ·  0/81 full</t>
+          <t xml:space="preserve">UMUT CAA CELLS  ·  umut  ·  81/81 full</t>
         </is>
       </c>
     </row>
@@ -436,6 +398,51 @@
           <t xml:space="preserve">A</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK ATP7B KO g3 p102</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK ATP7B KO g3 p99</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK ATP7B KO g3 p97</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK TOX4 OX p+12</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK TOX4 OX p+3</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK TOX4 OX p+3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK TOX4 OX p+4</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK TOX4 OX p+4</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR NT KO p?</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -443,6 +450,51 @@
           <t xml:space="preserve">B</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2 p?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2 p?</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2 p?</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR ATP7B KO p?</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR ATF3 KO p?</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR+1 p?</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2 p?</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2 p?</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR+1 p?</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -450,6 +502,51 @@
           <t xml:space="preserve">C</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 p50</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 TOX4 OX p+3</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 CBX3 KO g2 p6</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 CBX3 KO g1 p6</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 p+2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 p+2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 p+2</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 gNT p6</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 HOXB6 KO g1 p6</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -457,6 +554,51 @@
           <t xml:space="preserve">D</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LCC-V p?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap V1G1 p+1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada CASPEX (no sort) p+20</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap ER p</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada V1G1 p+2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canadaa V1G1 p+1</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canadaa V1G1 p+1</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada p+11</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada CASPEX (no sort) p+20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -464,6 +606,51 @@
           <t xml:space="preserve">E</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR NT KO p?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR MTF1 KO p?</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR ATP7B KO p?</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2 p?</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR MTF1 KO p?</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR+1 p?</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuPar50CR ATF3 KO p?</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p+8</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -471,6 +658,51 @@
           <t xml:space="preserve">F</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR p11</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR p9</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR p11</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR p9</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR p11</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR p11</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUCX gP1 p20</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUCX gP1 p20</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR p11</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -478,6 +710,51 @@
           <t xml:space="preserve">G</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada CASPEX (no sort) p+20</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada p+15</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada p+15</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada p+6</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada V1G1 p+2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada p+15</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LCC-V 99.17% p?</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX gNT p+21</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX gP1 p+21</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -485,11 +762,101 @@
           <t xml:space="preserve">H</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK FOXA1 KO g2 p16</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK JUN1 KO g2 p13</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK RFX KO g2 p17</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK FOXA1 KO g1 p17</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK HOXB6 KO g1 p18</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK RFX KO g1 p17</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK SPEN KO g2 p14</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK HOXB6 KO g2 p18</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK FOXA1 KO g1 p14</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
           <t xml:space="preserve">I</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK GATA6 KO g2 p18</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK NRF2 KO g1 p17</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK NRF2 KO g2 p17</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK FOXA1 KO g2 p14</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK GATA6 KO g1 p18</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK CBX3 KO G1 p15</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK POU3F3 KO g1 p15</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK ATP7B-GFP p47</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK gNT (10) p15</t>
         </is>
       </c>
     </row>
@@ -503,14 +870,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CAA CELLS  ·  umut  ·  81/81 full</t>
+          <t xml:space="preserve">UMUT CELLS -80  ·  umut  ·  81/81 full</t>
         </is>
       </c>
     </row>
@@ -570,47 +937,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3 p102</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1 p4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3 p99</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1 p4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3 p97</t>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p?</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX p+12</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT p+6</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX p+3</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT p+6</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX p+3</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX p+4</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3 p+7</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX p+4</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1 p5</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO p?</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+7</t>
         </is>
       </c>
     </row>
@@ -622,47 +989,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2 p?</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1 p28</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2 p?</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1 p28</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2 p?</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 p28</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO p?</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 p28</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO p?</t>
+          <t xml:space="preserve">HEK JUN KO g1 p19</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR+1 p?</t>
+          <t xml:space="preserve">HEK STAT1 KO g2 p30</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2 p?</t>
+          <t xml:space="preserve">HEK STAT1 KO g1 p19</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2 p?</t>
+          <t xml:space="preserve">HEK SMARCE1 KO g2 p19</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR+1 p?</t>
+          <t xml:space="preserve">HEK SMARCE1 KO g1 p19</t>
         </is>
       </c>
     </row>
@@ -674,47 +1041,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 p50</t>
+          <t xml:space="preserve">HEK293T p14</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 OX p+3</t>
+          <t xml:space="preserve">HEK293T p19</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 KO g2 p6</t>
+          <t xml:space="preserve">HEK APEX1 g1 p19</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 KO g1 p6</t>
+          <t xml:space="preserve">HEK STAT1 KO g2 p28</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 p+2</t>
+          <t xml:space="preserve">HEK gNT(20) p13</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 p+2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1 p13</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 p+2</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 p13</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT p6</t>
+          <t xml:space="preserve">HEK 3xFLAG p+6</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 HOXB6 KO g1 p6</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2 p37</t>
         </is>
       </c>
     </row>
@@ -726,47 +1093,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V p?</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3 p+9</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap V1G1 p+1</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1 p7</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX (no sort) p+20</t>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p|+7</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap ER p</t>
+          <t xml:space="preserve">Du145 p11</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G1 p+2</t>
+          <t xml:space="preserve">Du145 p11</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canadaa V1G1 p+1</t>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p+9</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canadaa V1G1 p+1</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT p14</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada p+11</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+12</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX (no sort) p+20</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3 p10</t>
         </is>
       </c>
     </row>
@@ -778,47 +1145,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO p?</t>
+          <t xml:space="preserve">Huh7 HOXB6 OX p6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO p?</t>
+          <t xml:space="preserve">Huh7 POU3F3 KO g1 p6</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO p?</t>
+          <t xml:space="preserve">Huh7 CBX3 OX p6</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2 p?</t>
+          <t xml:space="preserve">Huh7 POU3F3 KO g2 p6</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO p?</t>
+          <t xml:space="preserve">Huh7 TOX4 KO p+12</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR+1 p?</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24 p82</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO p?</t>
+          <t xml:space="preserve">Huh7 TOX4 KO g1 p?</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p+8</t>
+          <t xml:space="preserve">Huh7 ATP7B KO p81</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24 p84</t>
         </is>
       </c>
     </row>
@@ -830,47 +1197,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR p11</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1 p48</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR p9</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1 p48</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR p11</t>
+          <t xml:space="preserve">HEK gNT p22</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR p9</t>
+          <t xml:space="preserve">HEK gNT p22</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR p11</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2 p37</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR p11</t>
+          <t xml:space="preserve">HEK ATP7B KO g3 p+7</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP1 p20</t>
+          <t xml:space="preserve">HEK TOX4 KO g2 p+6</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP1 p20</t>
+          <t xml:space="preserve">HEK TOX4 KO g2 p+7</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR p11</t>
+          <t xml:space="preserve">HEK293T p19</t>
         </is>
       </c>
     </row>
@@ -882,47 +1249,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX (no sort) p+20</t>
+          <t xml:space="preserve">LNCX gNT p+20</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada p+15</t>
+          <t xml:space="preserve">LNCX gNT p+20</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada p+15</t>
+          <t xml:space="preserve">LNCX gP2 p+21</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada p+6</t>
+          <t xml:space="preserve">LNCX gP2 p+20</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G1 p+2</t>
+          <t xml:space="preserve">LnCap Canada V1G4 p41</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada p+15</t>
+          <t xml:space="preserve">LnCap Canada V1G3 p41</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17% p?</t>
+          <t xml:space="preserve">LnCap Canada V1G2 p41</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT p+21</t>
+          <t xml:space="preserve">LnCapCASPEX no select E p45769</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP1 p+21</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #1 p?</t>
         </is>
       </c>
     </row>
@@ -934,47 +1301,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2 p16</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1 p43</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN1 KO g2 p13</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX p42</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK RFX KO g2 p17</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1 p43</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1 p17</t>
+          <t xml:space="preserve">HEK ATP7B GFP p42</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1 p18</t>
+          <t xml:space="preserve">HEK ATP7B GFP p42</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK RFX KO g1 p17</t>
+          <t xml:space="preserve">HEK CASPEX gNT p?</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SPEN KO g2 p14</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX p42</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g2 p18</t>
+          <t xml:space="preserve">HEK APEX1 OX p21</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1 p14</t>
+          <t xml:space="preserve">HEK CBX3 OX p28</t>
         </is>
       </c>
     </row>
@@ -986,47 +1353,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK GATA6 KO g2 p18</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK NRF2 KO g1 p17</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+4</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK NRF2 KO g2 p17</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+4</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2 p14</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+4</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK GATA6 KO g1 p18</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+4</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO G1 p15</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1 p15</t>
+          <t xml:space="preserve">Du145 p?</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B-GFP p47</t>
+          <t xml:space="preserve">DuPar50CR+1 p218</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT (10) p15</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3 p8</t>
         </is>
       </c>
     </row>
@@ -1040,14 +1407,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -80  ·  umut  ·  81/81 full</t>
+          <t xml:space="preserve">DUZENLE  ·  umut  ·  74/81 full</t>
         </is>
       </c>
     </row>
@@ -1107,47 +1474,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1 p4</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1 p10</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1 p4</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3 p10</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1 p10</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p+2</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Du145 p25</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Du145 p25</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuDtxR p14</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuDtxR p14</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p?</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT p+6</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT p+6</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+5</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3 p+7</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1 p5</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+7</t>
         </is>
       </c>
     </row>
@@ -1159,47 +1526,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1 p28</t>
+          <t xml:space="preserve">LnCapCASPEX no select p?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1 p28</t>
+          <t xml:space="preserve">LnCapCASPEX no select C p?</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 p28</t>
+          <t xml:space="preserve">LnCapCASPEX no select E p?</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 p28</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #2 p?</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN KO g1 p19</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #2 p?</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2 p30</t>
+          <t xml:space="preserve">LnCapCASPEX no select H p?</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g1 p19</t>
+          <t xml:space="preserve">LnCapCASPEX no select H p?</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SMARCE1 KO g2 p19</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #1 p?</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SMARCE1 KO g1 p19</t>
+          <t xml:space="preserve">LCC-K no sort p?</t>
         </is>
       </c>
     </row>
@@ -1211,47 +1578,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T p14</t>
+          <t xml:space="preserve">LCC-I no sort p?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T p19</t>
+          <t xml:space="preserve">LCC-R no sort p?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 g1 p19</t>
+          <t xml:space="preserve">LCC-V no sort p?</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2 p28</t>
+          <t xml:space="preserve">LCC-C* p?</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20) p13</t>
+          <t xml:space="preserve">LCC-H p?</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1 p13</t>
+          <t xml:space="preserve">LCC-E p?</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 p13</t>
+          <t xml:space="preserve">LCC-K p?</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG p+6</t>
+          <t xml:space="preserve">LCC-I p?</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2 p37</t>
+          <t xml:space="preserve">LCC-K p?</t>
         </is>
       </c>
     </row>
@@ -1263,47 +1630,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3 p+9</t>
+          <t xml:space="preserve">LCC-R p?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1 p7</t>
+          <t xml:space="preserve">LCC-I p?</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p|+7</t>
+          <t xml:space="preserve">LCC-R p?</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 p11</t>
+          <t xml:space="preserve">LnCap Canada V1G1 p?</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 p11</t>
+          <t xml:space="preserve">LnCap Canada V1G1 p?</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p+9</t>
+          <t xml:space="preserve">LnCap Canada V1G1 p?</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT p14</t>
+          <t xml:space="preserve">LnCap Canada V1G1 p?</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+12</t>
+          <t xml:space="preserve">LNCX p+21</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3 p10</t>
+          <t xml:space="preserve">LNCX p+21</t>
         </is>
       </c>
     </row>
@@ -1315,47 +1682,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 HOXB6 OX p6</t>
+          <t xml:space="preserve">Huh7 POU3F2 KO g1 p?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F3 KO g1 p6</t>
+          <t xml:space="preserve">Huh7 TOX4 KO p+15</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 OX p6</t>
+          <t xml:space="preserve">Huh7 TOX4 KO p+14</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F3 KO g2 p6</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep2 p13</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 KO p+12</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24 p82</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 TOX4 KO g1 p?</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 ATP7B KO p81</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24 p84</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep2 p14</t>
         </is>
       </c>
     </row>
@@ -1367,47 +1714,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1 p48</t>
+          <t xml:space="preserve">HEK TOX4 KO g2 p+9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1 p48</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 p40</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT p22</t>
+          <t xml:space="preserve">HEK APEX1 KO g2 p22</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT p22</t>
+          <t xml:space="preserve">HEK ATP7B-GFP p30</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2 p37</t>
+          <t xml:space="preserve">HEK JUN KO g2 p18</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3 p+7</t>
+          <t xml:space="preserve">HEK E2F1 sh2 p20</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 KO g2 p+6</t>
+          <t xml:space="preserve">HEK ATP7B-GFP p30</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 KO g2 p+7</t>
+          <t xml:space="preserve">HEK E2F1 sh2 p20</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T p19</t>
+          <t xml:space="preserve">HEK ATP7B-GFP p30</t>
         </is>
       </c>
     </row>
@@ -1419,47 +1766,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT p+20</t>
+          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use) p+11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT p+20</t>
+          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use) p+11</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP2 p+21</t>
+          <t xml:space="preserve">LnCap Canada p+9</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP2 p+20</t>
+          <t xml:space="preserve">LnCap Canada p+9</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G4 p41</t>
+          <t xml:space="preserve">LNCX p+21</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G3 p41</t>
+          <t xml:space="preserve">LNCX p+21</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G2 p41</t>
+          <t xml:space="preserve">LNCX gP1 p+24</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select E p45769</t>
+          <t xml:space="preserve">LNCX gP2 p+25</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #1 p?</t>
+          <t xml:space="preserve">LNCX gP2 p+25</t>
         </is>
       </c>
     </row>
@@ -1471,47 +1818,37 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1 p43</t>
+          <t xml:space="preserve">LuCap35CR p11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX p42</t>
+          <t xml:space="preserve">LUCX p15</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1 p43</t>
+          <t xml:space="preserve">LUCX p15</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B GFP p42</t>
+          <t xml:space="preserve">LUCX p17</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B GFP p42</t>
+          <t xml:space="preserve">LUCX p17</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX gNT p?</t>
+          <t xml:space="preserve">LUCX p17</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX p42</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK APEX1 OX p21</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK CBX3 OX p28</t>
+          <t xml:space="preserve">LUCX p19</t>
         </is>
       </c>
     </row>
@@ -1523,47 +1860,42 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+3</t>
+          <t xml:space="preserve">HEK E2F1 sh1 p20</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+4</t>
+          <t xml:space="preserve">HEK ATP7B-GFP p31</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+4</t>
+          <t xml:space="preserve">HEK E2F1 sh1 p20</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+4</t>
+          <t xml:space="preserve">HEK ATP7B-GFP p31</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+4</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 plv-GFP p42</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 p+4</t>
+          <t xml:space="preserve">HEK ATP7B KO g3 p+2</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 p?</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuPar50CR+1 p218</t>
+          <t xml:space="preserve">HEK ATP7B KO g3 p+2</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3 p8</t>
+          <t xml:space="preserve">HEK ATF3 OX rep2 p24</t>
         </is>
       </c>
     </row>
@@ -1577,14 +1909,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DUZENLE  ·  umut  ·  74/81 full</t>
+          <t xml:space="preserve">ONGOING  ·  umut  ·  76/81 full</t>
         </is>
       </c>
     </row>
@@ -1644,47 +1976,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1 p10</t>
+          <t xml:space="preserve">LNCX p+22</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3 p10</t>
+          <t xml:space="preserve">LCC-V 99.17% p+4</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1 p10</t>
+          <t xml:space="preserve">LnCap478 #2 98% p28</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p+2</t>
+          <t xml:space="preserve">LnCap Canada p+7</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 p25</t>
+          <t xml:space="preserve">LnCap (m3) no sort p+14</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 p25</t>
+          <t xml:space="preserve">LnCap Canada p+14</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR p14</t>
+          <t xml:space="preserve">LnCap (m3) (sortER) p+13</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR p14</t>
+          <t xml:space="preserve">LnCap (m3) (sortER) p+13</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2 p?</t>
+          <t xml:space="preserve">LnCap Canada p+14</t>
         </is>
       </c>
     </row>
@@ -1696,47 +2028,47 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select p?</t>
+          <t xml:space="preserve">HEK TOX4 OX 3xFLAG p2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select C p?</t>
+          <t xml:space="preserve">HEK293T p7</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select E p?</t>
+          <t xml:space="preserve">HEK gNT(20) p16</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #2 p?</t>
+          <t xml:space="preserve">HEK ATF3 KO 20 p18</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #2 p?</t>
+          <t xml:space="preserve">HEK 3xFLAG p+7</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select H p?</t>
+          <t xml:space="preserve">HEK HOXB6 OX p36</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select H p?</t>
+          <t xml:space="preserve">HEK lef1 OX p?</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #1 p?</t>
+          <t xml:space="preserve">HEK ATF3 OX p?</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-K no sort p?</t>
+          <t xml:space="preserve">HEK ATP7B KO g3 p+13</t>
         </is>
       </c>
     </row>
@@ -1748,47 +2080,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-I no sort p?</t>
+          <t xml:space="preserve">Huh7 lef1 OX p?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-R no sort p?</t>
+          <t xml:space="preserve">Huh7 3xFLAG p?</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V no sort p?</t>
+          <t xml:space="preserve">Huh7 CASPEX gNT p?</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-C* p?</t>
+          <t xml:space="preserve">Huh7 ATF3 KO20 p6</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-H p?</t>
+          <t xml:space="preserve">Huh7 ATF3 OX20r1 p6</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-E p?</t>
+          <t xml:space="preserve">Huh7 ATF3KO10 p7</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-K p?</t>
+          <t xml:space="preserve">Huh7 p51</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-I p?</t>
+          <t xml:space="preserve">Huh7 p51</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-K p?</t>
+          <t xml:space="preserve">Huh7 p42</t>
         </is>
       </c>
     </row>
@@ -1800,47 +2132,47 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-R p?</t>
+          <t xml:space="preserve">HEK HOXB6 OX p36</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-I p?</t>
+          <t xml:space="preserve">HEK ATF3 OX10r1 p18</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-R p?</t>
+          <t xml:space="preserve">HEK ATP7B KO-1 p11</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G1 p?</t>
+          <t xml:space="preserve">HEK ATP7B KO-2 p11</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G1 p?</t>
+          <t xml:space="preserve">HEK ATP7B KO-3 p11</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G1 p?</t>
+          <t xml:space="preserve">HEK ATP7B GFP p53</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G1 p?</t>
+          <t xml:space="preserve">HEK ATF3 KO10 p9</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX p+21</t>
+          <t xml:space="preserve">HEK CASPEX Single p+6</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX p+21</t>
+          <t xml:space="preserve">HEK CASPEX Single p+6</t>
         </is>
       </c>
     </row>
@@ -1852,27 +2184,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F2 KO g1 p?</t>
+          <t xml:space="preserve">HepG2 p+2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 KO p+15</t>
+          <t xml:space="preserve">HepG2 p+2</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 KO p+14</t>
+          <t xml:space="preserve">HepG2 p+5</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep2 p13</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep2 p14</t>
+          <t xml:space="preserve">HepG2 p7</t>
         </is>
       </c>
     </row>
@@ -1884,47 +2211,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 KO g2 p+9</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT p?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 p40</t>
+          <t xml:space="preserve">Du145 p14</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 KO g2 p22</t>
+          <t xml:space="preserve">Du145 ATF3 KO rep2 p14</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B-GFP p30</t>
+          <t xml:space="preserve">Du145 ATF3 OX rep2 p14</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN KO g2 p18</t>
+          <t xml:space="preserve">Du145 p?</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2 p20</t>
+          <t xml:space="preserve">Du145 p?</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B-GFP p30</t>
+          <t xml:space="preserve">Du145 p?</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2 p20</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1 p15</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B-GFP p30</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT p+3</t>
         </is>
       </c>
     </row>
@@ -1936,47 +2263,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use) p+11</t>
+          <t xml:space="preserve">LnCap Canada p+23</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use) p+11</t>
+          <t xml:space="preserve">LNCAP BMK p?</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada p+9</t>
+          <t xml:space="preserve">LnCap Canada p+17</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada p+9</t>
+          <t xml:space="preserve">LnCap Canada p+17</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX p+21</t>
+          <t xml:space="preserve">LnCap Canada p+17</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX p+21</t>
+          <t xml:space="preserve">LnCap Canada p+17</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP1 p+24</t>
+          <t xml:space="preserve">LNC478 #2 98% p24</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP2 p+25</t>
+          <t xml:space="preserve">LNC478 #1 p23</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP2 p+25</t>
+          <t xml:space="preserve">LNC478 #3 p23</t>
         </is>
       </c>
     </row>
@@ -1988,37 +2315,47 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t xml:space="preserve">LuCap35CR p9</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap (m1) no sort p10</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR p10</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t xml:space="preserve">LuCap35CR p11</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX p15</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX p15</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX p17</t>
-        </is>
-      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX p17</t>
+          <t xml:space="preserve">LuCap35CR p11</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX p17</t>
+          <t xml:space="preserve">LUCX gP2 p20</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX p19</t>
+          <t xml:space="preserve">LUCX gP1 p20</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUCX gP1 p20</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUCX gP2 p20</t>
         </is>
       </c>
     </row>
@@ -2030,42 +2367,47 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1 p20</t>
+          <t xml:space="preserve">LnCap Canada p+14</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B-GFP p31</t>
+          <t xml:space="preserve">LNCX p12</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1 p20</t>
+          <t xml:space="preserve">LNCX p+17</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B-GFP p31</t>
+          <t xml:space="preserve">LNCX p+17</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 plv-GFP p42</t>
+          <t xml:space="preserve">LnCap Canada p+14</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3 p+2</t>
+          <t xml:space="preserve">LnCap Canada p+14</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3 p+2</t>
+          <t xml:space="preserve">LNCX gNT p+24</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX gP2 p+24</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep2 p24</t>
+          <t xml:space="preserve">LNCX gP1 p+24</t>
         </is>
       </c>
     </row>
@@ -2079,14 +2421,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ONGOING  ·  umut  ·  76/81 full</t>
+          <t xml:space="preserve">UMUT CELLS -4-  ·  umut  ·  30/81 full</t>
         </is>
       </c>
     </row>
@@ -2146,47 +2488,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX p+22</t>
+          <t xml:space="preserve">HEK ATF3 OX20r1 p18</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17% p+4</t>
+          <t xml:space="preserve">HEK ATF3OX10r1 p6</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap478 #2 98% p28</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada p+7</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap (m3) no sort p+14</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada p+14</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap (m3) (sortER) p+13</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap (m3) (sortER) p+13</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada p+14</t>
+          <t xml:space="preserve">HEK gNT p27</t>
         </is>
       </c>
     </row>
@@ -2198,47 +2510,37 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX 3xFLAG p2</t>
+          <t xml:space="preserve">HEK293T p14</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T p7</t>
+          <t xml:space="preserve">HEK293T p14</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20) p16</t>
+          <t xml:space="preserve">HEK293T p21</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO 20 p18</t>
+          <t xml:space="preserve">HEK293T p16</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG p+7</t>
+          <t xml:space="preserve">HEK293T p13</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX p36</t>
+          <t xml:space="preserve">HEK293T p16</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK lef1 OX p?</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATF3 OX p?</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATP7B KO g3 p+13</t>
+          <t xml:space="preserve">HEK293T p14</t>
         </is>
       </c>
     </row>
@@ -2250,47 +2552,47 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 lef1 OX p?</t>
+          <t xml:space="preserve">Du145 p10</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG p?</t>
+          <t xml:space="preserve">Du145 p10</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CASPEX gNT p?</t>
+          <t xml:space="preserve">Du145 p10</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO20 p6</t>
+          <t xml:space="preserve">Du145 p10</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX20r1 p6</t>
+          <t xml:space="preserve">Du145 p11</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3KO10 p7</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT p+3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 p51</t>
+          <t xml:space="preserve">Du145 p11</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 p51</t>
+          <t xml:space="preserve">Du145 p11</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 p42</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3 p15</t>
         </is>
       </c>
     </row>
@@ -2302,47 +2604,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX p36</t>
+          <t xml:space="preserve">Huh7 p51</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX10r1 p18</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATP7B KO-1 p11</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATP7B KO-2 p11</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATP7B KO-3 p11</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATP7B GFP p53</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATF3 KO10 p9</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK CASPEX Single p+6</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK CASPEX Single p+6</t>
+          <t xml:space="preserve">Huh7 p15</t>
         </is>
       </c>
     </row>
@@ -2354,22 +2621,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HepG2 p+2</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 p?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HepG2 p+2</t>
+          <t xml:space="preserve">DuDtxR CASPEXe g3 p15</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HepG2 p+5</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1 p15</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HepG2 p7</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 (eski) p?</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 (eski) p?</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1 (eski) p?</t>
         </is>
       </c>
     </row>
@@ -2381,47 +2658,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT p?</t>
+          <t xml:space="preserve">MDA-MB g1.1 p10 p10</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 p14</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 ATF3 KO rep2 p14</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 ATF3 OX rep2 p14</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 p?</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 p?</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 p?</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1 p15</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT p+3</t>
+          <t xml:space="preserve">MDA-MB gNT p10</t>
         </is>
       </c>
     </row>
@@ -2433,47 +2675,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada p+23</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCAP BMK p?</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada p+17</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada p+17</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada p+17</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada p+17</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNC478 #2 98% p24</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNC478 #1 p23</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNC478 #3 p23</t>
+          <t xml:space="preserve">LNCX p19</t>
         </is>
       </c>
     </row>
@@ -2483,101 +2685,11 @@
           <t xml:space="preserve">H</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR p9</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap (m1) no sort p10</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR p10</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR p11</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR p11</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX gP2 p20</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX gP1 p20</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX gP1 p20</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX gP2 p20</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
           <t xml:space="preserve">I</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada p+14</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX p12</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX p+17</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX p+17</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada p+14</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada p+14</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX gNT p+24</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX gP2 p+24</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX gP1 p+24</t>
         </is>
       </c>
     </row>
@@ -2591,14 +2703,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1 → Rack 1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-  ·  umut  ·  30/81 full</t>
+          <t xml:space="preserve">Unnamed box  ·  umut  ·  0/81 full</t>
         </is>
       </c>
     </row>
@@ -2656,288 +2768,6 @@
           <t xml:space="preserve">A</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATF3 OX20r1 p18</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK ATF3OX10r1 p6</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK gNT p27</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">B</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T p14</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T p14</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T p21</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T p16</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T p13</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T p16</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T p14</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 p10</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 p10</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 p10</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 p10</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 p11</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT p+3</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 p11</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145 p11</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3 p15</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">D</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 p51</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7 p15</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">E</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 p?</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEXe g3 p15</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1 p15</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 (eski) p?</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 (eski) p?</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1 (eski) p?</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">F</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MDA-MB g1.1 p10 p10</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MDA-MB gNT p10</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">G</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX p19</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">H</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">I</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not placed yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unnamed box  ·  umut  ·  0/81 full</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">

</xml_diff>